<commit_message>
[Fix Data] Toto 캐릭터 Id 수정 및 BasicCostumeId 데이터 제거
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Character.xlsx
+++ b/JsonConverter/ExcelFiles/Character.xlsx
@@ -19,15 +19,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
   <x:si>
-    <x:t>character_selly_01</x:t>
+    <x:t>캐릭터 고유 ID</x:t>
   </x:si>
   <x:si>
-    <x:t>토토</x:t>
+    <x:t>Description</x:t>
   </x:si>
   <x:si>
-    <x:t>Id</x:t>
+    <x:t>Character_Toto_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>웰빙리아국의 왕자 루이를 구하기 위해&lt;nl&gt;위험한 모험에 나선 여전사.</x:t>
   </x:si>
   <x:si>
     <x:t>Hp</x:t>
@@ -36,31 +39,22 @@
     <x:t>int</x:t>
   </x:si>
   <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
+    <x:t>토토</x:t>
+  </x:si>
+  <x:si>
     <x:t>Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string</x:t>
   </x:si>
   <x:si>
     <x:t>(name)</x:t>
   </x:si>
   <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
     <x:t>캐릭터 전체 컨셉이나 스토리</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BasicCostumeId</x:t>
-  </x:si>
-  <x:si>
-    <x:t>캐릭터 고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Description</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Costume_03</x:t>
-  </x:si>
-  <x:si>
-    <x:t>웰빙리아국의 왕자 루이를 구하기 위해&lt;nl&gt;위험한 모험에 나선 여전사.</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -153,7 +147,7 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="3">
+  <x:borders count="2">
     <x:border>
       <x:left>
         <x:color auto="1"/>
@@ -182,27 +176,13 @@
         <x:color auto="1"/>
       </x:bottom>
     </x:border>
-    <x:border>
-      <x:left style="thin">
-        <x:color rgb="ff000000"/>
-      </x:left>
-      <x:right style="thin">
-        <x:color rgb="ff000000"/>
-      </x:right>
-      <x:top style="thin">
-        <x:color rgb="ff000000"/>
-      </x:top>
-      <x:bottom style="thin">
-        <x:color rgb="ff000000"/>
-      </x:bottom>
-    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <x:alignment horizontal="general" vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="15">
+  <x:cellXfs count="13">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:alignment horizontal="general" vertical="center"/>
     </x:xf>
@@ -241,12 +221,6 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="general" vertical="bottom"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="general" vertical="bottom"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="bottom"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -858,70 +832,61 @@
     <x:col min="1" max="1" width="19.453125" style="2" customWidth="1"/>
     <x:col min="2" max="2" width="19.54296875" style="2" customWidth="1"/>
     <x:col min="3" max="3" width="72" style="2" customWidth="1"/>
-    <x:col min="4" max="4" width="26.54296875" style="2" customWidth="1"/>
-    <x:col min="5" max="7" width="12.54296875" style="2" bestFit="1" customWidth="1"/>
+    <x:col min="4" max="7" width="12.54296875" style="2" bestFit="1" customWidth="1"/>
     <x:col min="8" max="16384" width="12.54296875" style="2"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:3" ht="15.75" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>10</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="1"/>
       <x:c r="C1" s="1" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:4" ht="13.199999999999999">
+      <x:c r="A2" s="1" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B2" s="1" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C2" s="1" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D2" s="2" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:4" s="12" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A3" s="11" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B3" s="11" t="s">
         <x:v>8</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" spans="1:5" ht="13.199999999999999">
-      <x:c r="A2" s="1" t="s">
-        <x:v>6</x:v>
+      <x:c r="C3" s="11" t="s">
+        <x:v>1</x:v>
       </x:c>
-      <x:c r="B2" s="1" t="s">
+      <x:c r="D3" s="12" t="s">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:15" ht="15.75" customHeight="1">
+      <x:c r="A4" s="3" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B4" s="3" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="C2" s="1" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D2" s="1" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="E2" s="2" t="s">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:5" s="12" customFormat="1" ht="15.75" customHeight="1">
-      <x:c r="A3" s="11" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B3" s="11" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C3" s="11" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="D3" s="13" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="E3" s="12" t="s">
+      <x:c r="C4" s="3" t="s">
         <x:v>3</x:v>
       </x:c>
-    </x:row>
-    <x:row r="4" spans="1:15" ht="15.75" customHeight="1">
-      <x:c r="A4" s="3" t="s">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="B4" s="3" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C4" s="3" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="D4" s="14" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="E4" s="4">
+      <x:c r="D4" s="4">
         <x:v>100</x:v>
       </x:c>
+      <x:c r="E4" s="4"/>
       <x:c r="F4" s="4"/>
       <x:c r="G4" s="4"/>
       <x:c r="H4" s="4"/>

</xml_diff>